<commit_message>
Doplnit M badge na play-off mistra v moderní éře (1986-2020/21)
Žádná moderní sezóna neměla M badge (mistr jen v META). Doplněn M na řádek
skutečného mistra = vítěze play-off (ne 1. místa ZČ) — řeší MASTER_REPORT nález #2:
- 2020/21 → Třinec (ne Sparta 1.ZČ), 2009/10 → Pardubice (ne Plzeň), 2008/09 → KV
  (ne Slavia), 2013/14 → Zlín, 2014/15 → Litvínov, 2017/18 → Kometa Brno…
- 1992/93 (poslední federální): mistr HC Sparta Praha (finále 3:1 Vítkovice; ověřeno
  webem — Litvínov byl 1.ZČ, vypadl v SF). 2019/20: bez titulu (COVID, play-off zrušeno).

Token-overlap matching META mistr ↔ tabulka. Všech 73 sezón s titulem má M na mistrovi.
</commit_message>
<xml_diff>
--- a/data/S1986_87_FINAL.xlsx
+++ b/data/S1986_87_FINAL.xlsx
@@ -719,6 +719,11 @@
           <t>Tesla Pardubice</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F4" t="n">
         <v>34</v>
       </c>
@@ -23485,7 +23490,6 @@
           <t>NODE_S1986_87_0009</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23606,8 +23610,6 @@
           <t>NODE_S1986_87_0007</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23663,8 +23665,6 @@
           <t>NODE_S1986_87_0007</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23720,8 +23720,6 @@
           <t>NODE_S1986_87_0007</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23777,8 +23775,6 @@
           <t>NODE_S1986_87_0007</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23834,8 +23830,6 @@
           <t>NODE_S1986_87_0001</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23891,8 +23885,6 @@
           <t>NODE_S1986_87_0007</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24123,8 +24115,6 @@
           <t>NODE_S1986_87_0004</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24175,8 +24165,6 @@
           <t>NODE_S1986_87_0004</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24227,8 +24215,6 @@
           <t>NODE_S1986_87_0004</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24630,8 +24616,6 @@
           <t>NODE_S1986_87_0027</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24729,8 +24713,6 @@
           <t>NODE_S1986_87_0027</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24974,8 +24956,6 @@
           <t>NODE_S1986_87_0033</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25172,8 +25152,6 @@
           <t>NODE_S1986_87_0039</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25229,8 +25207,6 @@
           <t>NODE_S1986_87_0039</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25286,8 +25262,6 @@
           <t>NODE_S1986_87_0040</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25343,8 +25317,6 @@
           <t>NODE_S1986_87_0040</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25400,8 +25372,6 @@
           <t>NODE_S1986_87_0038</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25462,7 +25432,6 @@
           <t>NODE_S1986_87_0051</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -25701,8 +25670,6 @@
           <t>NODE_S1986_87_0046</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26082,7 +26049,6 @@
           <t>NODE_S1986_87_0060</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26138,8 +26104,6 @@
           <t>NODE_S1986_87_0057</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26401,8 +26365,6 @@
           <t>NODE_S1986_87_0062</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26453,8 +26415,6 @@
           <t>NODE_S1986_87_0062</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26646,8 +26606,6 @@
           <t>NODE_S1986_87_0062</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26904,8 +26862,6 @@
           <t>NODE_S1986_87_0072</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -26956,8 +26912,6 @@
           <t>NODE_S1986_87_0072</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27196,8 +27150,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27248,8 +27200,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27300,8 +27250,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27352,8 +27300,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
       <c r="I85" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27404,8 +27350,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27456,8 +27400,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
       <c r="I87" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27508,8 +27450,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27560,8 +27500,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27612,8 +27550,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -27664,8 +27600,6 @@
           <t>NODE_S1986_87_0078</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -28292,8 +28226,6 @@
           <t>NODE_S1986_87_0092</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -28344,8 +28276,6 @@
           <t>NODE_S1986_87_0092</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -28396,8 +28326,6 @@
           <t>NODE_S1986_87_0092</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -28448,8 +28376,6 @@
           <t>NODE_S1986_87_0092</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -28500,8 +28426,6 @@
           <t>NODE_S1986_87_0092</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -28552,8 +28476,6 @@
           <t>NODE_S1986_87_0092</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -28745,7 +28667,6 @@
           <t>NODE_S1986_87_0111</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
           <t>NODE_S1986_87_0115</t>
@@ -28848,8 +28769,6 @@
           <t>NODE_S1986_87_0111</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -29276,7 +29195,6 @@
           <t>NODE_S1986_87_0125</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -29327,8 +29245,6 @@
           <t>NODE_S1986_87_0129</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -29379,8 +29295,6 @@
           <t>NODE_S1986_87_0004</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -29557,8 +29471,6 @@
           <t>NODE_S1986_87_0129</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -58640,7 +58552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58844,6 +58756,18 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>II.SNHL finále: první utkání doma; do kvalifikace o 2. SNHL sestoupila Levoča; TJ Spartak BEZ Bratislava přímo do KP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>mistr</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Tesla Pardubice</t>
         </is>
       </c>
     </row>

</xml_diff>